<commit_message>
[FEAT] - cập nhật chức năng thời khóa biểu và table động
</commit_message>
<xml_diff>
--- a/public/template_cham_cong_export.xlsx
+++ b/public/template_cham_cong_export.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\presonal\Programming\VsCode\PersonalProjects\APIStudents\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B49F20-C46F-433C-86C5-6DB204370622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E2AE5E-728D-4B93-BE6C-5B3E57B97251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -526,12 +526,33 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -550,15 +571,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -591,18 +603,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1445,13 +1445,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
       <c r="F1" s="27"/>
       <c r="G1" s="28"/>
     </row>
@@ -1465,15 +1465,15 @@
       <c r="G2" s="28"/>
     </row>
     <row r="3" spans="1:7" ht="25" x14ac:dyDescent="0.35">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="4" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A4" s="30"/>
@@ -2238,7 +2238,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81DEFBB4-68C6-4C20-94D3-81BC97A8A25F}">
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" style="4" customWidth="1"/>
@@ -2251,8 +2251,8 @@
     <col min="9" max="9" width="17.7265625" style="4" customWidth="1"/>
     <col min="10" max="10" width="16.81640625" style="4" customWidth="1"/>
     <col min="11" max="11" width="16.90625" style="4" customWidth="1"/>
-    <col min="12" max="12" width="14.1796875" style="4" customWidth="1"/>
-    <col min="13" max="256" width="9.1796875" style="4"/>
+    <col min="12" max="13" width="14.1796875" style="4" customWidth="1"/>
+    <col min="14" max="256" width="9.1796875" style="4"/>
     <col min="257" max="257" width="7" style="4" customWidth="1"/>
     <col min="258" max="258" width="29.54296875" style="4" customWidth="1"/>
     <col min="259" max="259" width="12.54296875" style="4" customWidth="1"/>
@@ -3011,76 +3011,76 @@
     <col min="16141" max="16384" width="9.1796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
     </row>
-    <row r="2" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="70" t="s">
+    <row r="2" spans="1:13" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-    </row>
-    <row r="3" spans="1:12" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="47" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+    </row>
+    <row r="3" spans="1:13" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="53" t="s">
+      <c r="D3" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="67" t="s">
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
+      <c r="M3" s="48" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="3" customFormat="1" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="48"/>
-      <c r="B4" s="51"/>
-      <c r="C4" s="48"/>
+    <row r="4" spans="1:13" s="3" customFormat="1" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="55"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="55"/>
       <c r="D4" s="5"/>
-      <c r="E4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="K4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="L4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="68"/>
-    </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="49"/>
-      <c r="B5" s="52"/>
-      <c r="C5" s="49"/>
+      <c r="M4" s="49"/>
+    </row>
+    <row r="5" spans="1:13" s="3" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="56"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="56"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="69"/>
-    </row>
-    <row r="6" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="7"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="50"/>
+    </row>
+    <row r="6" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -3094,7 +3094,7 @@
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
     </row>
-    <row r="7" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -3108,7 +3108,7 @@
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="8" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -3122,7 +3122,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
     </row>
-    <row r="9" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -3136,7 +3136,7 @@
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
     </row>
-    <row r="10" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -3150,7 +3150,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
     </row>
-    <row r="11" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -3164,7 +3164,7 @@
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
     </row>
-    <row r="12" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -3178,7 +3178,7 @@
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
     </row>
-    <row r="13" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -3192,7 +3192,7 @@
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
     </row>
-    <row r="14" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -3206,7 +3206,7 @@
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
     </row>
-    <row r="15" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -3220,7 +3220,7 @@
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
     </row>
-    <row r="16" spans="1:12" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -3341,13 +3341,11 @@
     <row r="70" ht="33.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="71" ht="21" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="4">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C3:C5"/>
-    <mergeCell ref="H3:H5"/>
-    <mergeCell ref="D3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="B3 B73:B65536">
     <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
@@ -3943,12 +3941,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="56"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="60"/>
       <c r="E1" s="9"/>
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
@@ -3956,17 +3954,17 @@
       <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="83.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
     </row>
     <row r="3" spans="1:9" ht="96.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
@@ -5687,26 +5685,26 @@
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
-      <c r="E1" s="62" t="s">
+      <c r="E1" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:9" ht="20" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="64" t="s">
+      <c r="B2" s="67"/>
+      <c r="C2" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="64"/>
-      <c r="E2" s="63" t="s">
+      <c r="D2" s="68"/>
+      <c r="E2" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
     </row>
     <row r="3" spans="1:9" ht="20.5" x14ac:dyDescent="0.35">
       <c r="A3" s="24"/>
@@ -5736,17 +5734,17 @@
       <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:9" ht="20.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="65"/>
-      <c r="B6" s="65"/>
-      <c r="C6" s="66" t="s">
+      <c r="A6" s="69"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="66"/>
-      <c r="E6" s="65" t="s">
+      <c r="D6" s="70"/>
+      <c r="E6" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
     </row>
     <row r="9" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A9" s="16"/>
@@ -5754,29 +5752,29 @@
       <c r="C9" s="40"/>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
-      <c r="F9" s="59" t="s">
+      <c r="F9" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
+      <c r="G9" s="63"/>
+      <c r="H9" s="63"/>
+      <c r="I9" s="63"/>
     </row>
     <row r="10" spans="1:9" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="60" t="s">
+      <c r="A10" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="60"/>
-      <c r="C10" s="60" t="s">
+      <c r="B10" s="64"/>
+      <c r="C10" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60" t="s">
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="64"/>
     </row>
     <row r="11" spans="1:9" ht="39.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="16"/>
@@ -5792,17 +5790,17 @@
     <row r="12" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A12" s="16"/>
       <c r="B12" s="17"/>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61" t="s">
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="65"/>
     </row>
     <row r="17" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A17" s="16"/>
@@ -5810,29 +5808,29 @@
       <c r="C17" s="26"/>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
-      <c r="F17" s="59" t="s">
+      <c r="F17" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
+      <c r="I17" s="63"/>
     </row>
     <row r="18" spans="1:9" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="60" t="s">
+      <c r="A18" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="60"/>
-      <c r="C18" s="60" t="s">
+      <c r="B18" s="64"/>
+      <c r="C18" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60" t="s">
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="60"/>
-      <c r="H18" s="60"/>
-      <c r="I18" s="60"/>
+      <c r="G18" s="64"/>
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
     </row>
     <row r="19" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A19" s="16"/>
@@ -5848,17 +5846,17 @@
     <row r="20" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61" t="s">
+      <c r="D20" s="65"/>
+      <c r="E20" s="65"/>
+      <c r="F20" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
-      <c r="I20" s="61"/>
+      <c r="G20" s="65"/>
+      <c r="H20" s="65"/>
+      <c r="I20" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>